<commit_message>
Update TestWeave test suite workbook
</commit_message>
<xml_diff>
--- a/testweave/test-suite.xlsx
+++ b/testweave/test-suite.xlsx
@@ -710,7 +710,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Passed</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Passed</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Passed</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Failed</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Failed: JDBC URL is required.</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Failed</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Passed (100 samples)</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Passed</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Passed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update VeyraAI test suite workbook
</commit_message>
<xml_diff>
--- a/testweave/test-suite.xlsx
+++ b/testweave/test-suite.xlsx
@@ -1081,12 +1081,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Registration Web Test</t>
+          <t>TestCase1 Performance Test</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t/>
+          <t>{"authorization":{"type":"None","token":""},"headers":{"Accept":"application/json","User-Agent":"API-Validator-Tool/1.0","Content-Type":"application/json"},"endpoint":"http://216.10.245.166/Library/GetBook.php?AuthorName=Sainath","method":"GET","requestFormat":"JSON","headersText":"Accept: application/json\nContent-Type: application/json\nUser-Agent: API-Validator-Tool/1.0","params":{"AuthorName":"Sainath"},"authType":"None"}</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1141,17 +1141,17 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>{"headless":false,"startUrl":"https://eventhub.rahulshettyacademy.com/login","stepType":"WEB_TEST","slowMoMillis":0,"steps":[{"note":"page loaded","suggested":false,"action":"Navigate","selector":"","value":"https://eventhub.rahulshettyacademy.com/login"},{"note":"Suggested after navigation","suggested":true,"action":"Validate Text","selector":"h2","value":"EventHub \u2014 Discover &amp; Book Events"},{"note":"Register","suggested":false,"action":"Click","selector":"a.text-indigo-600.hover\\:underline","value":""},{"note":"","suggested":false,"action":"Click","selector":"[data-testid=\"register-email\"]","value":""},{"note":"","suggested":false,"action":"Type","selector":"[data-testid=\"register-email\"]","value":"sai5611@live.in"},{"note":"","suggested":false,"action":"Click","selector":"[data-testid=\"register-password\"]","value":""},{"note":"password input","suggested":false,"action":"Type","selector":"[data-testid=\"register-password\"]","value":"Sai@ss15031993"},{"note":"","suggested":false,"action":"Click","selector":"[placeholder=\"Repeat\\ your\\ password\"]","value":""},{"note":"password input","suggested":false,"action":"Type","selector":"[placeholder=\"Repeat\\ your\\ password\"]","value":"Sai@ss15031993"},{"note":"Create Account","suggested":false,"action":"Click","selector":"[data-testid=\"register-btn\"]","value":""},{"note":"Logout","suggested":false,"action":"Click","selector":"[data-testid=\"logout-btn\"]","value":""},{"note":"","suggested":false,"action":"Click","selector":"#email","value":""},{"note":"","suggested":false,"action":"Type","selector":"#email","value":"sai5611@live.in"},{"note":"","suggested":false,"action":"Click","selector":"#password","value":""},{"note":"password input","suggested":false,"action":"Type","selector":"#password","value":"Sai@ss15031993"},{"note":"Sign In","suggested":false,"action":"Click","selector":"#login-btn","value":""},{"note":"Logout","suggested":false,"action":"Click","selector":"[data-testid=\"logout-btn\"]","value":""}],"testName":"RegistrationFlow"}</t>
+          <t/>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t/>
+          <t>{"stepType":"PERFORMANCE_TEST","iterationsPerThread":10,"threads":10,"requestBodySource":"Performance Test"}</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Failed (8 failed)</t>
+          <t>Passed (100 samples)</t>
         </is>
       </c>
     </row>
@@ -1178,12 +1178,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TestCase1 Performance Test</t>
+          <t>WebUI</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>{"authorization":{"type":"None","token":""},"headers":{"Accept":"application/json","User-Agent":"API-Validator-Tool/1.0","Content-Type":"application/json"},"endpoint":"http://216.10.245.166/Library/GetBook.php?AuthorName=Sainath","method":"GET","requestFormat":"JSON","headersText":"Accept: application/json\nContent-Type: application/json\nUser-Agent: API-Validator-Tool/1.0","params":{"AuthorName":"Sainath"},"authType":"None"}</t>
+          <t/>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>{}</t>
+          <t/>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1238,12 +1238,12 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t/>
+          <t>{"headless":true,"startUrl":"https://eventhub.rahulshettyacademy.com/login","stepType":"WEB_TEST","slowMoMillis":0,"steps":[{"note":"page loaded","flowVariableName":"","stepName":"Navigate page loaded","action":"Navigate","step":"1","selector":"","value":"https://eventhub.rahulshettyacademy.com/login","timeout":""},{"note":"Correct Flow Variable syntax while preserving unique reusable email","flowVariableName":"email","stepName":"Flow Variable email","action":"Flow Variable","step":"2","selector":"email","value":"sai${randomInt}@live.in","timeout":""},{"note":"Healed Get Text selector to uniquely target the visible EventHub heading","flowVariableName":"","stepName":"Get Text EventHub Practice App","action":"Get Text","step":"3","selector":"text=\"EventHub \u2014 Practice App\"","value":"EventHub \u2014 Practice App","timeout":""},{"note":"Register","flowVariableName":"","stepName":"Click a text-indigo-600 hover underline","action":"Click","step":"4","selector":"a.text-indigo-600.hover\\:underline","value":"","timeout":""},{"note":"","flowVariableName":"","stepName":"Click register-email","action":"Click","step":"5","selector":"[data-testid=\"register-email\"]","value":"","timeout":""},{"note":"","flowVariableName":"","stepName":"Type register-email","action":"Type","step":"6","selector":"[data-testid=\"register-email\"]","value":"${email}","timeout":""},{"note":"","flowVariableName":"","stepName":"Click register-password","action":"Click","step":"7","selector":"[data-testid=\"register-password\"]","value":"","timeout":""},{"note":"password input","flowVariableName":"","stepName":"Type register-password","action":"Type","step":"8","selector":"[data-testid=\"register-password\"]","value":"Sai@ss15031993","timeout":""},{"note":"","flowVariableName":"","stepName":"Click Repeat your password","action":"Click","step":"9","selector":"[placeholder=\"Repeat\\ your\\ password\"]","value":"","timeout":""},{"note":"password input","flowVariableName":"","stepName":"Type Repeat your password","action":"Type","step":"10","selector":"[placeholder=\"Repeat\\ your\\ password\"]","value":"Sai@ss15031993","timeout":""},{"note":"Create Account","flowVariableName":"","stepName":"Click register-btn","action":"Click","step":"11","selector":"[data-testid=\"register-btn\"]","value":"","timeout":""},{"note":"Logout","flowVariableName":"","stepName":"Click logout-btn","action":"Click","step":"12","selector":"[data-testid=\"logout-btn\"]","value":"","timeout":""},{"note":"","flowVariableName":"","stepName":"Click email","action":"Click","step":"13","selector":"#email","value":"","timeout":""},{"note":"","flowVariableName":"","stepName":"Type email","action":"Type","step":"14","selector":"#email","value":"${email}","timeout":""},{"note":"","flowVariableName":"","stepName":"Click password","action":"Click","step":"15","selector":"#password","value":"","timeout":""},{"note":"password input","flowVariableName":"","stepName":"Type password","action":"Type","step":"16","selector":"#password","value":"Sai@ss15031993","timeout":""},{"note":"Sign In","flowVariableName":"","stepName":"Click login-btn","action":"Click","step":"17","selector":"#login-btn","value":"","timeout":""},{"note":"Logout","flowVariableName":"","stepName":"Click logout-btn","action":"Click","step":"18","selector":"[data-testid=\"logout-btn\"]","value":"","timeout":""}],"testName":"RegistrationFlow"}</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>{"stepType":"PERFORMANCE_TEST","iterationsPerThread":10,"threads":10,"requestBodySource":"Performance Test"}</t>
+          <t/>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Passed (100 samples)</t>
+          <t>Passed</t>
         </is>
       </c>
     </row>

</xml_diff>